<commit_message>
Replace S2 with the verified-note version and add the completed PRISMA 2020 checklist
</commit_message>
<xml_diff>
--- a/docs/supplementary/Supplementary_Table_S2_fulltext_exclusions.xlsx
+++ b/docs/supplementary/Supplementary_Table_S2_fulltext_exclusions.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="450" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="279">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -480,7 +480,7 @@
     <t xml:space="preserve">IEEE Internet of Things Journal</t>
   </si>
   <si>
-    <t xml:space="preserve">Wisconsin Breast Cancer (FNA cytology image-derived) + Fetal Health (CTG signal); used as tabular benchmarks, no image processing -- image-derived, trio definitional call</t>
+    <t xml:space="preserve">Wisconsin Breast Cancer (FNA cytology, image-derived) and Fetal Health (CTG signal) used as tabular benchmarks, with no image processing.</t>
   </si>
   <si>
     <t xml:space="preserve">10.1109/tce.2025.3548303</t>
@@ -624,7 +624,7 @@
     <t xml:space="preserve">Traitement du Signal</t>
   </si>
   <si>
-    <t xml:space="preserve">mixed benchmark: natural + aerial + medical images; general FRQI edge-detection, medical use incidental -- protocol §5.3 open decision</t>
+    <t xml:space="preserve">Mixed benchmark of natural, aerial and medical images for general FRQI edge detection. Medical use is incidental.</t>
   </si>
   <si>
     <t xml:space="preserve">10.3390/biom12111576</t>
@@ -639,7 +639,7 @@
     <t xml:space="preserve">Biomolecules</t>
   </si>
   <si>
-    <t xml:space="preserve">ImageNet ants/bees (non-medical images) + Wisconsin Breast Cancer (FNA cytology-derived, but tabular); primary image dataset is non-medical -&gt; excludable regardless</t>
+    <t xml:space="preserve">ImageNet ants/bees (non-medical images) and Wisconsin Breast Cancer (FNA cytology-derived, tabular). The primary image dataset is non-medical.</t>
   </si>
   <si>
     <t xml:space="preserve">10.3934/math.2025499</t>
@@ -711,7 +711,7 @@
     <t xml:space="preserve">Patterns</t>
   </si>
   <si>
-    <t xml:space="preserve">reads as perspective; task=other, no dataset [GUESS: confirm in abstract]</t>
+    <t xml:space="preserve">Perspective article (type confirmed on the journal page). No primary dataset.</t>
   </si>
   <si>
     <t xml:space="preserve">10.1038/s41585-025-01058-y</t>
@@ -726,7 +726,7 @@
     <t xml:space="preserve">Nature Reviews Urology</t>
   </si>
   <si>
-    <t xml:space="preserve">reads as perspective ('quantum leap'); task=other, no dataset [GUESS]</t>
+    <t xml:space="preserve">Comment article of two pages (type confirmed on the journal page). No primary dataset.</t>
   </si>
   <si>
     <t xml:space="preserve">10.1109/access.2022.3195044</t>
@@ -753,7 +753,7 @@
     <t xml:space="preserve">Technology in Cancer Research &amp; Treatment</t>
   </si>
   <si>
-    <t xml:space="preserve">reads as review; task=other, no dataset [GUESS]</t>
+    <t xml:space="preserve">Review article (literature review of nine studies, as stated in its abstract). No primary dataset.</t>
   </si>
   <si>
     <t xml:space="preserve">10.3390/medsci12040067</t>
@@ -768,7 +768,7 @@
     <t xml:space="preserve">Medical Sciences</t>
   </si>
   <si>
-    <t xml:space="preserve">reads as overview; task=other, no dataset [GUESS]</t>
+    <t xml:space="preserve">Review article (type confirmed on the publisher page). No primary dataset.</t>
   </si>
   <si>
     <t xml:space="preserve">10.7759/cureus.67486</t>
@@ -783,6 +783,9 @@
     <t xml:space="preserve">Cureus</t>
   </si>
   <si>
+    <t xml:space="preserve">Narrative review (type stated in its abstract). No primary dataset.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Supplementary Table S2. Reports excluded at full text (N = 48), with reason, exclusion route and recorded basis</t>
   </si>
   <si>
@@ -811,6 +814,9 @@
   </si>
   <si>
     <t xml:space="preserve">All sources are in the public repository https://github.com/lpapp-muw/qc-medimaging-review. Titles and journals come from the full-text extraction workbook, and years from the co-author extraction.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eight reviewer notes were reworded before publication on 25 September 2026: for five secondary articles the article type was confirmed on the journal, publisher or abstract page, and three notes had internal working remarks removed. The original notes remain in the repository CSV.</t>
   </si>
   <si>
     <t xml:space="preserve">"Reason as recorded" is the exclusion reason exactly as stored. "Reason (consolidated)" groups it into the nine categories reported in Section III-A. "Recorded note" is the note stored with each decision: the rule inputs for the automated route, and the reviewer note for the individual reviews.</t>
@@ -2863,7 +2869,7 @@
         <v>84</v>
       </c>
       <c r="J49" s="2" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -2884,7 +2890,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -2892,12 +2898,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2905,17 +2911,17 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2923,32 +2929,37 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>264</v>
       </c>
     </row>
   </sheetData>
@@ -2980,33 +2991,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D2" s="6" t="n">
         <f aca="false">COUNTA(S2_fulltext_exclusions!$B$2:$B$49)</f>
@@ -3022,7 +3033,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>6</v>
@@ -3044,7 +3055,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>6</v>
@@ -3066,7 +3077,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>6</v>
@@ -3088,7 +3099,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>7</v>
@@ -3198,7 +3209,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>7</v>
@@ -3242,7 +3253,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>7</v>

</xml_diff>